<commit_message>
Phase 2: fix CUDA cu128 env, add B0 shutdown script & annotations
- Update run_phase2_ablation.sh to use .venv-5090 (cu128, sm_120 support)
- Add run_B0_and_shutdown.sh for standalone B0 training
- Add market1501/msmt17 annotation files
- Add dataset attribute definitions
- Update phase2 experiment tracker xlsx
</commit_message>
<xml_diff>
--- a/docs/experiments/phase2_ablation_results.xlsx
+++ b/docs/experiments/phase2_ablation_results.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase2 Ablation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="历史结果参考" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统一配置" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Phase2 Ablation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="历史结果参考" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="统一配置" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,11 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM"/>
+    <numFmt numFmtId="166" formatCode="YYYY-MM-DD HH:MM"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -121,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -167,7 +166,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -733,8 +735,8 @@
       <c r="I4" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="J4" s="17" t="n">
-        <v>46060.73828672147</v>
+      <c r="J4" s="18" t="n">
+        <v>46063.49705296653</v>
       </c>
       <c r="L4" s="10">
         <f>IF(AND(K4&lt;&gt;"",J4&lt;&gt;""),(K4-J4)*24,"")</f>
@@ -1187,12 +1189,12 @@
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="G2:I2"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="J2:L2"/>
     <mergeCell ref="A1:S1"/>
-    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="M2:P2"/>
     <mergeCell ref="C2:F2"/>
-    <mergeCell ref="G2:I2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:P2"/>
     <mergeCell ref="Q2:S2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: sync remaining local updates and annotations
</commit_message>
<xml_diff>
--- a/docs/experiments/phase2_ablation_results.xlsx
+++ b/docs/experiments/phase2_ablation_results.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Phase2 Ablation" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="历史结果参考" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="统一配置" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase2 Ablation" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="历史结果参考" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统一配置" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -172,6 +172,12 @@
     <xf numFmtId="166" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -537,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -736,19 +742,26 @@
         <v>60</v>
       </c>
       <c r="J4" s="18" t="n">
-        <v>46063.49705296653</v>
+        <v>46063.49705296296</v>
+      </c>
+      <c r="K4" s="19" t="n">
+        <v>46063.58682533565</v>
       </c>
       <c r="L4" s="10">
         <f>IF(AND(K4&lt;&gt;"",J4&lt;&gt;""),(K4-J4)*24,"")</f>
         <v/>
       </c>
-      <c r="M4" s="11" t="n"/>
-      <c r="N4" s="11" t="n"/>
+      <c r="M4" s="11" t="n">
+        <v>0.8420000000000001</v>
+      </c>
+      <c r="N4" s="11" t="n">
+        <v>0.9279999999999999</v>
+      </c>
       <c r="O4" s="11" t="n"/>
       <c r="P4" s="11" t="n"/>
       <c r="R4" s="9" t="inlineStr">
         <is>
-          <t>运行中</t>
+          <t>已完成</t>
         </is>
       </c>
     </row>
@@ -790,17 +803,22 @@
       <c r="I5" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="J5" s="12" t="inlineStr">
-        <is>
-          <t>复用B0的Stage1 checkpoint</t>
-        </is>
+      <c r="J5" s="20" t="n">
+        <v>46063.58683628472</v>
+      </c>
+      <c r="K5" s="19" t="n">
+        <v>46063.63456403935</v>
       </c>
       <c r="L5" s="13">
         <f>IF(AND(K5&lt;&gt;"",J5&lt;&gt;""),(K5-J5)*24,"")</f>
         <v/>
       </c>
-      <c r="M5" s="11" t="n"/>
-      <c r="N5" s="11" t="n"/>
+      <c r="M5" s="11" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="N5" s="11" t="n">
+        <v>0.9320000000000001</v>
+      </c>
       <c r="O5" s="11" t="n"/>
       <c r="P5" s="11" t="n"/>
       <c r="Q5" s="11">
@@ -809,7 +827,7 @@
       </c>
       <c r="R5" s="12" t="inlineStr">
         <is>
-          <t>待运行</t>
+          <t>已完成</t>
         </is>
       </c>
     </row>
@@ -851,17 +869,22 @@
       <c r="I6" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="J6" s="9" t="inlineStr">
-        <is>
-          <t>复用B0的Stage1 checkpoint</t>
-        </is>
+      <c r="J6" s="18" t="n">
+        <v>46063.634576875</v>
+      </c>
+      <c r="K6" s="19" t="n">
+        <v>46063.68180732639</v>
       </c>
       <c r="L6" s="10">
         <f>IF(AND(K6&lt;&gt;"",J6&lt;&gt;""),(K6-J6)*24,"")</f>
         <v/>
       </c>
-      <c r="M6" s="11" t="n"/>
-      <c r="N6" s="11" t="n"/>
+      <c r="M6" s="11" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="N6" s="11" t="n">
+        <v>0.9390000000000001</v>
+      </c>
       <c r="O6" s="11" t="n"/>
       <c r="P6" s="11" t="n"/>
       <c r="Q6" s="14">
@@ -870,7 +893,7 @@
       </c>
       <c r="R6" s="9" t="inlineStr">
         <is>
-          <t>待运行</t>
+          <t>已完成</t>
         </is>
       </c>
     </row>
@@ -912,17 +935,22 @@
       <c r="I7" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>复用B0的Stage1 checkpoint</t>
-        </is>
+      <c r="J7" s="20" t="n">
+        <v>46063.68181951389</v>
+      </c>
+      <c r="K7" s="19" t="n">
+        <v>46063.72891876158</v>
       </c>
       <c r="L7" s="13">
         <f>IF(AND(K7&lt;&gt;"",J7&lt;&gt;""),(K7-J7)*24,"")</f>
         <v/>
       </c>
-      <c r="M7" s="11" t="n"/>
-      <c r="N7" s="11" t="n"/>
+      <c r="M7" s="11" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="N7" s="11" t="n">
+        <v>0.9379999999999999</v>
+      </c>
       <c r="O7" s="11" t="n"/>
       <c r="P7" s="11" t="n"/>
       <c r="Q7" s="11">
@@ -931,7 +959,7 @@
       </c>
       <c r="R7" s="12" t="inlineStr">
         <is>
-          <t>待运行</t>
+          <t>已完成</t>
         </is>
       </c>
     </row>
@@ -973,17 +1001,22 @@
       <c r="I8" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="J8" s="9" t="inlineStr">
-        <is>
-          <t>复用B0的Stage1, 同B0但Stage2重训</t>
-        </is>
+      <c r="J8" s="18" t="n">
+        <v>46063.72893152778</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>46063.77614086805</v>
       </c>
       <c r="L8" s="10">
         <f>IF(AND(K8&lt;&gt;"",J8&lt;&gt;""),(K8-J8)*24,"")</f>
         <v/>
       </c>
-      <c r="M8" s="11" t="n"/>
-      <c r="N8" s="11" t="n"/>
+      <c r="M8" s="11" t="n">
+        <v>0.8440000000000001</v>
+      </c>
+      <c r="N8" s="11" t="n">
+        <v>0.9309999999999999</v>
+      </c>
       <c r="O8" s="11" t="n"/>
       <c r="P8" s="11" t="n"/>
       <c r="Q8" s="14">
@@ -992,7 +1025,7 @@
       </c>
       <c r="R8" s="9" t="inlineStr">
         <is>
-          <t>待运行</t>
+          <t>已完成</t>
         </is>
       </c>
     </row>
@@ -1034,17 +1067,22 @@
       <c r="I9" s="12" t="n">
         <v>60</v>
       </c>
-      <c r="J9" s="12" t="inlineStr">
-        <is>
-          <t>复用B0的Stage1 checkpoint</t>
-        </is>
+      <c r="J9" s="20" t="n">
+        <v>46063.77615399306</v>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>46063.82345755787</v>
       </c>
       <c r="L9" s="13">
         <f>IF(AND(K9&lt;&gt;"",J9&lt;&gt;""),(K9-J9)*24,"")</f>
         <v/>
       </c>
-      <c r="M9" s="11" t="n"/>
-      <c r="N9" s="11" t="n"/>
+      <c r="M9" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N9" s="11" t="n">
+        <v>0.9159999999999999</v>
+      </c>
       <c r="O9" s="11" t="n"/>
       <c r="P9" s="11" t="n"/>
       <c r="Q9" s="11">
@@ -1053,7 +1091,7 @@
       </c>
       <c r="R9" s="12" t="inlineStr">
         <is>
-          <t>待运行</t>
+          <t>已完成</t>
         </is>
       </c>
     </row>
@@ -1095,17 +1133,22 @@
       <c r="I10" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="J10" s="9" t="inlineStr">
-        <is>
-          <t>Stage1+Stage2 全量训练 (query_encoder)</t>
-        </is>
+      <c r="J10" s="18" t="n">
+        <v>46063.82347071759</v>
+      </c>
+      <c r="K10" s="19" t="n">
+        <v>46063.9140759375</v>
       </c>
       <c r="L10" s="10">
         <f>IF(AND(K10&lt;&gt;"",J10&lt;&gt;""),(K10-J10)*24,"")</f>
         <v/>
       </c>
-      <c r="M10" s="11" t="n"/>
-      <c r="N10" s="11" t="n"/>
+      <c r="M10" s="11" t="n">
+        <v>0.865</v>
+      </c>
+      <c r="N10" s="11" t="n">
+        <v>0.9390000000000001</v>
+      </c>
       <c r="O10" s="11" t="n"/>
       <c r="P10" s="11" t="n"/>
       <c r="Q10" s="14">
@@ -1114,7 +1157,7 @@
       </c>
       <c r="R10" s="9" t="inlineStr">
         <is>
-          <t>待运行</t>
+          <t>已完成</t>
         </is>
       </c>
     </row>
@@ -1184,6 +1227,67 @@
       <c r="R11" s="12" t="inlineStr">
         <is>
           <t>待运行</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B3a最优 + SIE + OLP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>clip_native</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>60</v>
+      </c>
+      <c r="I12" t="n">
+        <v>60</v>
+      </c>
+      <c r="J12" s="19" t="n">
+        <v>46063.96574074074</v>
+      </c>
+      <c r="K12" s="19" t="n">
+        <v>46064.00050925926</v>
+      </c>
+      <c r="L12" s="21" t="n">
+        <v>0.8344444444444444</v>
+      </c>
+      <c r="M12" s="22" t="n">
+        <v>0.888</v>
+      </c>
+      <c r="N12" s="22" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="O12" s="22" t="n"/>
+      <c r="P12" s="22" t="n"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>已完成</t>
         </is>
       </c>
     </row>

</xml_diff>